<commit_message>
Add voice assistant Excel updates and multi-roll command support
</commit_message>
<xml_diff>
--- a/intelligent_voice_assistant/database/student_marks.xlsx
+++ b/intelligent_voice_assistant/database/student_marks.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,13 +484,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
         <v>30</v>
@@ -504,7 +504,7 @@
         <v>30</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
         <v>10</v>
@@ -518,7 +518,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
         <v>40</v>
@@ -532,7 +532,7 @@
         <v>50</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
         <v>8</v>
@@ -549,7 +549,7 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
@@ -563,7 +563,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -574,7 +574,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="D8" t="n">
         <v>8</v>
@@ -588,7 +588,7 @@
         <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
@@ -619,7 +619,7 @@
         <v>30</v>
       </c>
       <c r="C11" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
         <v>10</v>
@@ -680,6 +680,9 @@
       <c r="A18" t="n">
         <v>18</v>
       </c>
+      <c r="C18" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -758,6 +761,9 @@
       <c r="A30" t="n">
         <v>30</v>
       </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
       <c r="D30" t="n">
         <v>15</v>
       </c>
@@ -766,6 +772,9 @@
       <c r="A31" t="n">
         <v>31</v>
       </c>
+      <c r="C31" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -877,6 +886,14 @@
       </c>
       <c r="C45" t="n">
         <v>97</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve voice marks entry and dashboard behavior
</commit_message>
<xml_diff>
--- a/intelligent_voice_assistant/database/student_marks.xlsx
+++ b/intelligent_voice_assistant/database/student_marks.xlsx
@@ -484,16 +484,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -501,13 +501,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -515,13 +518,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
         <v>40</v>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -529,7 +535,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>10</v>
@@ -538,7 +544,7 @@
         <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -546,13 +552,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
         <v>18</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -560,10 +569,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>80</v>
+        <v>9</v>
+      </c>
+      <c r="E7" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -579,6 +591,9 @@
       <c r="D8" t="n">
         <v>8</v>
       </c>
+      <c r="E8" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -593,22 +608,25 @@
       <c r="D9" t="n">
         <v>3</v>
       </c>
+      <c r="E9" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="n">
         <v>20</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -616,16 +634,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
         <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12">
@@ -633,16 +651,25 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>23</v>
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>15</v>
       </c>
       <c r="D12" t="n">
         <v>32</v>
+      </c>
+      <c r="E12" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>12</v>
       </c>
+      <c r="B13" t="n">
+        <v>20</v>
+      </c>
       <c r="D13" t="n">
         <v>30</v>
       </c>
@@ -652,7 +679,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15">
@@ -767,6 +794,9 @@
       <c r="D30" t="n">
         <v>15</v>
       </c>
+      <c r="E30" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -830,6 +860,12 @@
       </c>
       <c r="B38" t="n">
         <v>30</v>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="39">

</xml_diff>